<commit_message>
Changed figure 1 and reorga
</commit_message>
<xml_diff>
--- a/data/SI/SI_2_site_selection.xlsx
+++ b/data/SI/SI_2_site_selection.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polymtlca-my.sharepoint.com/personal/marin_pellan_polymtl_ca/Documents/POST_DOC/CODE/regionalized_lci_mineral/data/SI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="371" documentId="8_{EF4B609D-3C32-4D85-B6D7-614095F206BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02ACB667-0E23-47D2-BBC6-8C0A7056C65F}"/>
+  <xr:revisionPtr revIDLastSave="373" documentId="8_{EF4B609D-3C32-4D85-B6D7-614095F206BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88FCCE22-8478-4D66-BAFC-621892BC3BE6}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B09C33A3-69AE-4EDE-B293-E9623AD2B114}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B09C33A3-69AE-4EDE-B293-E9623AD2B114}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="4" r:id="rId1"/>
@@ -3028,6 +3028,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B231D443-D3C4-4EF0-BDC9-8F5B03D7CAA5}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:DR68"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3182,7 +3183,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:38" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:38" s="7" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>45</v>
       </c>
@@ -3261,7 +3262,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:38" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:38" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>56</v>
       </c>
@@ -3425,7 +3426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>72</v>
       </c>
@@ -3516,7 +3517,7 @@
         <v>29.039084533163262</v>
       </c>
     </row>
-    <row r="6" spans="1:38" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:38" s="7" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>76</v>
       </c>
@@ -3596,7 +3597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>81</v>
       </c>
@@ -3687,7 +3688,7 @@
         <v>3.5165997959183577</v>
       </c>
     </row>
-    <row r="8" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>84</v>
       </c>
@@ -3861,7 +3862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>101</v>
       </c>
@@ -3955,7 +3956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>107</v>
       </c>
@@ -4049,7 +4050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>109</v>
       </c>
@@ -4140,7 +4141,7 @@
         <v>24.008283837755101</v>
       </c>
     </row>
-    <row r="13" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>112</v>
       </c>
@@ -4228,7 +4229,7 @@
         <v>2.7760508515306124</v>
       </c>
     </row>
-    <row r="14" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>114</v>
       </c>
@@ -4319,7 +4320,7 @@
         <v>7.7388999209183664</v>
       </c>
     </row>
-    <row r="15" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>116</v>
       </c>
@@ -4407,7 +4408,7 @@
         <v>0.12428704693877551</v>
       </c>
     </row>
-    <row r="16" spans="1:38" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:38" s="18" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
         <v>119</v>
       </c>
@@ -4497,7 +4498,7 @@
         <v>1.4536125510204081</v>
       </c>
     </row>
-    <row r="17" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>122</v>
       </c>
@@ -4585,7 +4586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>127</v>
       </c>
@@ -4679,7 +4680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>129</v>
       </c>
@@ -4770,7 +4771,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>135</v>
       </c>
@@ -4864,7 +4865,7 @@
         <v>4.4745421183166938</v>
       </c>
     </row>
-    <row r="21" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>140</v>
       </c>
@@ -4952,7 +4953,7 @@
         <v>4.476523630102041</v>
       </c>
     </row>
-    <row r="22" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
         <v>142</v>
       </c>
@@ -5120,7 +5121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>153</v>
       </c>
@@ -5208,7 +5209,7 @@
         <v>4.1704080612244905</v>
       </c>
     </row>
-    <row r="25" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
         <v>155</v>
       </c>
@@ -5305,7 +5306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
         <v>164</v>
       </c>
@@ -5399,7 +5400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
         <v>169</v>
       </c>
@@ -5490,7 +5491,7 @@
         <v>1.2201776096938775</v>
       </c>
     </row>
-    <row r="28" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
         <v>171</v>
       </c>
@@ -5581,7 +5582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:38" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
         <v>176</v>
       </c>
@@ -5672,7 +5673,7 @@
         <v>7.932820721938775</v>
       </c>
     </row>
-    <row r="30" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
         <v>178</v>
       </c>
@@ -5846,7 +5847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
         <v>189</v>
       </c>
@@ -5934,7 +5935,7 @@
         <v>7.253304461734694</v>
       </c>
     </row>
-    <row r="33" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
         <v>191</v>
       </c>
@@ -6022,7 +6023,7 @@
         <v>1.0473627551020408</v>
       </c>
     </row>
-    <row r="34" spans="1:38" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:38" s="7" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>193</v>
       </c>
@@ -6102,7 +6103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
         <v>199</v>
       </c>
@@ -6184,7 +6185,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
         <v>205</v>
       </c>
@@ -6275,7 +6276,7 @@
         <v>12.41413683010194</v>
       </c>
     </row>
-    <row r="37" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
         <v>207</v>
       </c>
@@ -6366,7 +6367,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
         <v>210</v>
       </c>
@@ -6457,7 +6458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
         <v>213</v>
       </c>
@@ -6545,7 +6546,7 @@
         <v>5.7128877551020407</v>
       </c>
     </row>
-    <row r="40" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
         <v>215</v>
       </c>
@@ -6636,7 +6637,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
         <v>217</v>
       </c>
@@ -6724,7 +6725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:38" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:38" s="7" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>220</v>
       </c>
@@ -6885,7 +6886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
         <v>231</v>
       </c>
@@ -6973,7 +6974,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
         <v>234</v>
       </c>
@@ -7067,7 +7068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
         <v>238</v>
       </c>
@@ -7155,7 +7156,7 @@
         <v>8.0534261301020305</v>
       </c>
     </row>
-    <row r="47" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
         <v>240</v>
       </c>
@@ -7249,7 +7250,7 @@
         <v>0.15869132653061224</v>
       </c>
     </row>
-    <row r="48" spans="1:38" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:38" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
         <v>243</v>
       </c>
@@ -7336,7 +7337,7 @@
         <v>3.5769025000000001</v>
       </c>
     </row>
-    <row r="49" spans="1:38" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:38" s="7" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
         <v>246</v>
       </c>
@@ -7416,7 +7417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
         <v>249</v>
       </c>
@@ -7590,7 +7591,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
         <v>257</v>
       </c>
@@ -7749,7 +7750,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
         <v>266</v>
       </c>
@@ -7837,7 +7838,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
         <v>270</v>
       </c>
@@ -7999,7 +8000,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
         <v>276</v>
       </c>
@@ -8087,7 +8088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="14" t="s">
         <v>279</v>
       </c>
@@ -8178,7 +8179,7 @@
         <v>4.1181668765306121</v>
       </c>
     </row>
-    <row r="59" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="14" t="s">
         <v>281</v>
       </c>
@@ -8266,7 +8267,7 @@
         <v>5.8747529081632548</v>
       </c>
     </row>
-    <row r="60" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="14"/>
       <c r="B60" t="s">
         <v>283</v>
@@ -8358,7 +8359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="14"/>
       <c r="B61" t="s">
         <v>289</v>
@@ -8450,7 +8451,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="14"/>
       <c r="B62" t="s">
         <v>290</v>
@@ -8542,7 +8543,7 @@
         <v>17.66760135719143</v>
       </c>
     </row>
-    <row r="63" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="14"/>
       <c r="B63" t="s">
         <v>293</v>
@@ -8631,7 +8632,7 @@
         <v>8.2519489795918357</v>
       </c>
     </row>
-    <row r="64" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="14"/>
       <c r="B64" t="s">
         <v>295</v>
@@ -8720,7 +8721,7 @@
         <v>4.2180154591836736</v>
       </c>
     </row>
-    <row r="65" spans="1:122" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:122" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="14"/>
       <c r="B65" t="s">
         <v>297</v>
@@ -8809,7 +8810,7 @@
         <v>1.2300799484693878</v>
       </c>
     </row>
-    <row r="66" spans="1:122" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:122" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="22"/>
       <c r="B66" s="23" t="s">
         <v>299</v>
@@ -9103,7 +9104,13 @@
       <c r="DR68" s="26"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:DR66" xr:uid="{B231D443-D3C4-4EF0-BDC9-8F5B03D7CAA5}"/>
+  <autoFilter ref="A1:DR66" xr:uid="{B231D443-D3C4-4EF0-BDC9-8F5B03D7CAA5}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="manufacturing"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>